<commit_message>
feat(automation): dedicated 18:00 WIB performance run (same-day close fill)
Adds .github/workflows/performance.yml on cron "0 11 * * 1-5" (18:00 WIB, Mon-Fri)
that runs ONLY the reporting layer after IDX close — the screener and evaluator.py
are untouched. New performance.run_performance_evening(): fetches OHLC for the
tickers awaiting evaluation with end=today+1 (yfinance end is exclusive, so the
standard incremental_update omits the current day), then runs the standard pass.
If the data source has published today's final bar, yesterday's signals are
evaluated on THIS run; otherwise rows stay pending and are backfilled on a later
run (never faked). Workflow restores the scan cache (read-only) and commits
data/performance/ to main. Morning 05:00 scan kept as-is.

Verified on real data: evening run fetched 2026-06-09 and evaluated the
2026-06-08 signals (swing 7/7, scalping 12/13) using 06-09 OHLC — same-day,
not postponed; 1 suspended-ticker row correctly left pending.
</commit_message>
<xml_diff>
--- a/data/performance/daily/signal_list_2026-06-08.xlsx
+++ b/data/performance/daily/signal_list_2026-06-08.xlsx
@@ -41,7 +41,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -74,6 +84,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +476,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Win Rate: 0.0%  (0W / 0L of 0 evaluated, 7 pending)</t>
+          <t>Win Rate: 57.1%  (4W / 3L of 7 evaluated)</t>
         </is>
       </c>
     </row>
@@ -531,11 +543,34 @@
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="C5" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2460</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -550,11 +585,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="C6" t="n">
+        <v>5925</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5950</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -569,11 +627,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
+      <c r="C7" t="n">
+        <v>7850</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8325</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8400</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -588,11 +669,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="C8" t="n">
+        <v>496</v>
+      </c>
+      <c r="D8" t="n">
+        <v>560</v>
+      </c>
+      <c r="E8" t="n">
+        <v>570</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -607,11 +711,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="C9" t="n">
+        <v>165</v>
+      </c>
+      <c r="D9" t="n">
+        <v>143</v>
+      </c>
+      <c r="E9" t="n">
+        <v>210</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>-13.33</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -626,11 +753,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="C10" t="n">
+        <v>113</v>
+      </c>
+      <c r="D10" t="n">
+        <v>106</v>
+      </c>
+      <c r="E10" t="n">
+        <v>113</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>-6.19</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -645,11 +795,34 @@
           <t>PRE_MARKUP</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="C11" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1095</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -689,7 +862,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Win Rate: 0.0%  (0W / 0L of 0 evaluated, 13 pending)</t>
+          <t>Win Rate: 41.7%  (5W / 7L of 12 evaluated, 1 pending)</t>
         </is>
       </c>
     </row>
@@ -756,11 +929,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="C5" t="n">
+        <v>246</v>
+      </c>
+      <c r="D5" t="n">
+        <v>252</v>
+      </c>
+      <c r="E5" t="n">
+        <v>286</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -775,11 +971,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="C6" t="n">
+        <v>6450</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6350</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6725</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -794,11 +1013,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
+      <c r="C7" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2460</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -813,11 +1055,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="C8" t="n">
+        <v>118</v>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" t="n">
+        <v>122</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>-11.02</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -832,11 +1097,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="C9" t="n">
+        <v>655</v>
+      </c>
+      <c r="D9" t="n">
+        <v>655</v>
+      </c>
+      <c r="E9" t="n">
+        <v>655</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -851,11 +1139,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="C10" t="n">
+        <v>266</v>
+      </c>
+      <c r="D10" t="n">
+        <v>270</v>
+      </c>
+      <c r="E10" t="n">
+        <v>278</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -870,11 +1181,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="C11" t="n">
+        <v>580</v>
+      </c>
+      <c r="D11" t="n">
+        <v>570</v>
+      </c>
+      <c r="E11" t="n">
+        <v>590</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>-1.72</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -889,11 +1223,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
+      <c r="C12" t="n">
+        <v>270</v>
+      </c>
+      <c r="D12" t="n">
+        <v>268</v>
+      </c>
+      <c r="E12" t="n">
+        <v>272</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -908,11 +1265,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="C13" t="n">
+        <v>169</v>
+      </c>
+      <c r="D13" t="n">
+        <v>191</v>
+      </c>
+      <c r="E13" t="n">
+        <v>226</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -927,11 +1307,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="C14" t="n">
+        <v>7850</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8325</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8400</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -946,8 +1349,21 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
+      <c r="C15" t="n">
+        <v/>
+      </c>
+      <c r="D15" t="n">
+        <v/>
+      </c>
+      <c r="E15" t="n">
+        <v/>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v/>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v/>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>pending</t>
@@ -965,11 +1381,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
+      <c r="C16" t="n">
+        <v>165</v>
+      </c>
+      <c r="D16" t="n">
+        <v>143</v>
+      </c>
+      <c r="E16" t="n">
+        <v>210</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>-13.33</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>
@@ -984,11 +1423,34 @@
           <t>SCALPING_HIGH</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
+      <c r="C17" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1095</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>evaluated</t>
         </is>
       </c>
     </row>

</xml_diff>